<commit_message>
Ajustes según reunión de fianzas
</commit_message>
<xml_diff>
--- a/Documentación/Brechas/brecha fianzas.xlsx
+++ b/Documentación/Brechas/brecha fianzas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\Documentación\Brechas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B5C29AB-E135-40D2-9C75-1BFA1E29995A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0315348-7D7D-4B9B-9BB3-93BB6C62ACB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{55631BAB-3F43-4C4D-BEDF-0998D0E484F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{55631BAB-3F43-4C4D-BEDF-0998D0E484F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Fianza - Emision" sheetId="3" r:id="rId1"/>
@@ -24,7 +24,6 @@
     <sheet name="Reportes matriz" sheetId="11" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -987,7 +986,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1087,17 +1086,14 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2157,54 +2153,54 @@
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="B29" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F29" s="6" t="s">
+      <c r="B29" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="E29" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="F29" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="G29" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="H29" s="10" t="s">
+      <c r="G29" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="H29" s="39" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F30" s="6" t="s">
+      <c r="B30" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="D30" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="G30" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="H30" s="10" t="s">
+      <c r="G30" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="H30" s="39" t="s">
         <v>108</v>
       </c>
     </row>
@@ -3421,54 +3417,54 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="27" t="s">
         <v>68</v>
       </c>
-      <c r="C5" s="37" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="F5" s="38" t="s">
+      <c r="C5" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="G5" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="H5" s="39" t="s">
+      <c r="G5" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" s="36" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="C6" s="37" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" s="38" t="s">
+      <c r="C6" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="G6" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="H6" s="40" t="s">
+      <c r="G6" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" s="30" t="s">
         <v>178</v>
       </c>
     </row>

</xml_diff>